<commit_message>
Updating load emulator v2
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/files/energy/input/load_emulator/input_emulator_v2/0. metadata_load_emulator_v2.xlsx
+++ b/files/energy/input/load_emulator/input_emulator_v2/0. metadata_load_emulator_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rsericerca-my.sharepoint.com/personal/rollo_rse-web_it/Documents/Desktop/CACER simulator - public repo/CACER-simulator/files/energy/input/load_emulator/input_emulator_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1040" documentId="11_F25DC773A252ABDACC1048A8291C5FB25ADE58F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5572848-43B9-46F0-8687-D788D81B3CCF}"/>
+  <xr:revisionPtr revIDLastSave="1049" documentId="11_F25DC773A252ABDACC1048A8291C5FB25ADE58F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA854FAF-612B-4940-B249-A39C593B9573}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="708" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="708" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clusters_distribution" sheetId="1" r:id="rId1"/>
@@ -86,7 +86,7 @@
     Dati Enea</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="4" shapeId="0" xr:uid="{95B473DF-5EA0-4072-B863-AB402273D0E4}">
+    <comment ref="J1" authorId="4" shapeId="0" xr:uid="{95B473DF-5EA0-4072-B863-AB402273D0E4}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -182,9 +182,6 @@
     <t>dishwasher</t>
   </si>
   <si>
-    <t>electric_hob</t>
-  </si>
-  <si>
     <t>iron</t>
   </si>
   <si>
@@ -282,6 +279,9 @@
   </si>
   <si>
     <t>cluster_percentage_normalized</t>
+  </si>
+  <si>
+    <t>induction_hob</t>
   </si>
 </sst>
 </file>
@@ -703,7 +703,7 @@
   <threadedComment ref="G1" dT="2026-03-24T14:26:12.90" personId="{776CA3F5-2BE0-4A02-A953-A7EBF94F0315}" id="{4C07C6BF-493D-48D0-8825-2913C57E620F}">
     <text>Dati Enea</text>
   </threadedComment>
-  <threadedComment ref="K1" dT="2026-03-24T14:27:18.28" personId="{776CA3F5-2BE0-4A02-A953-A7EBF94F0315}" id="{95B473DF-5EA0-4072-B863-AB402273D0E4}">
+  <threadedComment ref="J1" dT="2026-03-24T14:27:18.28" personId="{776CA3F5-2BE0-4A02-A953-A7EBF94F0315}" id="{95B473DF-5EA0-4072-B863-AB402273D0E4}">
     <text>Dati Enea e Istat integrati</text>
   </threadedComment>
   <threadedComment ref="O1" dT="2026-03-24T14:28:03.09" personId="{776CA3F5-2BE0-4A02-A953-A7EBF94F0315}" id="{DC63A6DC-43FB-4AF7-BDD1-B0933EF8579D}">
@@ -763,10 +763,10 @@
         <v>0</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
@@ -793,7 +793,7 @@
         <v>0.334610472541507</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I2" s="8"/>
       <c r="J2" s="9"/>
@@ -822,7 +822,7 @@
         <v>0.10089399744572157</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I3" s="8"/>
       <c r="J3" s="9"/>
@@ -851,7 +851,7 @@
         <v>8.9399744572158352E-2</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="9"/>
@@ -880,7 +880,7 @@
         <v>8.0459770114942514E-2</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="9"/>
@@ -909,7 +909,7 @@
         <v>8.0459770114942514E-2</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
@@ -936,7 +936,7 @@
         <v>7.6628352490421436E-2</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
@@ -963,7 +963,7 @@
         <v>7.2796934865900373E-2</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
@@ -990,7 +990,7 @@
         <v>6.3856960408684535E-2</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
@@ -1017,7 +1017,7 @@
         <v>5.1085568326947627E-2</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
@@ -1044,7 +1044,7 @@
         <v>4.9808429118773936E-2</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1073,8 +1073,9 @@
     <col min="2" max="5" width="12.77734375" customWidth="1"/>
     <col min="6" max="6" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="13" width="12.77734375" customWidth="1"/>
-    <col min="14" max="14" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="12.77734375" customWidth="1"/>
+    <col min="13" max="13" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="12.77734375" customWidth="1"/>
     <col min="18" max="18" width="19.44140625" bestFit="1" customWidth="1"/>
@@ -1093,97 +1094,97 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="V1" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="X1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Z1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="AB1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="AG1" s="1" t="s">
         <v>7</v>
@@ -1218,19 +1219,19 @@
         <v>0</v>
       </c>
       <c r="J2" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0.19</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0.99</v>
+      </c>
+      <c r="M2" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N2" s="2">
         <v>0.13</v>
-      </c>
-      <c r="K2" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="L2" s="2">
-        <v>0.19</v>
-      </c>
-      <c r="M2" s="2">
-        <v>0.99</v>
-      </c>
-      <c r="N2" s="2">
-        <v>0.28000000000000003</v>
       </c>
       <c r="O2" s="2">
         <v>0.85</v>
@@ -1319,19 +1320,19 @@
         <v>0.02</v>
       </c>
       <c r="J3" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0.99</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N3" s="2">
         <v>0.19</v>
-      </c>
-      <c r="K3" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="L3" s="2">
-        <v>0.15</v>
-      </c>
-      <c r="M3" s="2">
-        <v>0.99</v>
-      </c>
-      <c r="N3" s="2">
-        <v>0.28000000000000003</v>
       </c>
       <c r="O3" s="2">
         <v>0.85</v>
@@ -1420,19 +1421,19 @@
         <v>0.12</v>
       </c>
       <c r="J4" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="L4" s="2">
+        <v>1</v>
+      </c>
+      <c r="M4" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N4" s="2">
         <v>0.33</v>
-      </c>
-      <c r="K4" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="L4" s="2">
-        <v>0.3</v>
-      </c>
-      <c r="M4" s="2">
-        <v>1</v>
-      </c>
-      <c r="N4" s="2">
-        <v>0.28000000000000003</v>
       </c>
       <c r="O4" s="2">
         <v>0.85</v>
@@ -1521,19 +1522,19 @@
         <v>0.05</v>
       </c>
       <c r="J5" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="K5" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="L5" s="2">
+        <v>1</v>
+      </c>
+      <c r="M5" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N5" s="2">
         <v>0.27</v>
-      </c>
-      <c r="K5" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="L5" s="2">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="M5" s="2">
-        <v>1</v>
-      </c>
-      <c r="N5" s="2">
-        <v>0.28000000000000003</v>
       </c>
       <c r="O5" s="2">
         <v>0.85</v>
@@ -1622,19 +1623,19 @@
         <v>0.06</v>
       </c>
       <c r="J6" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0.37</v>
+      </c>
+      <c r="L6" s="2">
+        <v>1</v>
+      </c>
+      <c r="M6" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N6" s="2">
         <v>0.21</v>
-      </c>
-      <c r="K6" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="L6" s="2">
-        <v>0.37</v>
-      </c>
-      <c r="M6" s="2">
-        <v>1</v>
-      </c>
-      <c r="N6" s="2">
-        <v>0.28000000000000003</v>
       </c>
       <c r="O6" s="2">
         <v>0.85</v>
@@ -1723,19 +1724,19 @@
         <v>0.01</v>
       </c>
       <c r="J7" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="K7" s="2">
+        <v>0.37</v>
+      </c>
+      <c r="L7" s="2">
+        <v>1</v>
+      </c>
+      <c r="M7" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N7" s="2">
         <v>0.19</v>
-      </c>
-      <c r="K7" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="L7" s="2">
-        <v>0.37</v>
-      </c>
-      <c r="M7" s="2">
-        <v>1</v>
-      </c>
-      <c r="N7" s="2">
-        <v>0.28000000000000003</v>
       </c>
       <c r="O7" s="2">
         <v>0.85</v>
@@ -1824,19 +1825,19 @@
         <v>0.01</v>
       </c>
       <c r="J8" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="L8" s="2">
+        <v>1</v>
+      </c>
+      <c r="M8" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N8" s="2">
         <v>0.15</v>
-      </c>
-      <c r="K8" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="L8" s="2">
-        <v>0.33</v>
-      </c>
-      <c r="M8" s="2">
-        <v>1</v>
-      </c>
-      <c r="N8" s="2">
-        <v>0.28000000000000003</v>
       </c>
       <c r="O8" s="2">
         <v>0.85</v>
@@ -1925,19 +1926,19 @@
         <v>0.09</v>
       </c>
       <c r="J9" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0.26</v>
+      </c>
+      <c r="L9" s="2">
+        <v>1</v>
+      </c>
+      <c r="M9" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N9" s="2">
         <v>0.28999999999999998</v>
-      </c>
-      <c r="K9" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="L9" s="2">
-        <v>0.26</v>
-      </c>
-      <c r="M9" s="2">
-        <v>1</v>
-      </c>
-      <c r="N9" s="2">
-        <v>0.28000000000000003</v>
       </c>
       <c r="O9" s="2">
         <v>0.85</v>
@@ -2026,19 +2027,19 @@
         <v>0.01</v>
       </c>
       <c r="J10" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0.18</v>
+      </c>
+      <c r="L10" s="2">
+        <v>1</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N10" s="2">
         <v>0.19</v>
-      </c>
-      <c r="K10" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="L10" s="2">
-        <v>0.18</v>
-      </c>
-      <c r="M10" s="2">
-        <v>1</v>
-      </c>
-      <c r="N10" s="2">
-        <v>0.28000000000000003</v>
       </c>
       <c r="O10" s="2">
         <v>0.85</v>
@@ -2127,19 +2128,19 @@
         <v>0.01</v>
       </c>
       <c r="J11" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0.19</v>
+      </c>
+      <c r="L11" s="2">
+        <v>1</v>
+      </c>
+      <c r="M11" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="N11" s="2">
         <v>0.1</v>
-      </c>
-      <c r="K11" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="L11" s="2">
-        <v>0.19</v>
-      </c>
-      <c r="M11" s="2">
-        <v>1</v>
-      </c>
-      <c r="N11" s="2">
-        <v>0.28000000000000003</v>
       </c>
       <c r="O11" s="2">
         <v>0.85</v>
@@ -2229,8 +2230,9 @@
     <col min="2" max="5" width="12.77734375" customWidth="1"/>
     <col min="6" max="6" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="13" width="12.77734375" customWidth="1"/>
-    <col min="14" max="14" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="12.77734375" customWidth="1"/>
+    <col min="13" max="13" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="12.77734375" customWidth="1"/>
     <col min="18" max="18" width="19.44140625" bestFit="1" customWidth="1"/>
@@ -2246,100 +2248,100 @@
   <sheetData>
     <row r="1" spans="1:33" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="V1" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="X1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Z1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="AB1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="AG1" s="1" t="s">
         <v>7</v>
@@ -2383,10 +2385,10 @@
         <v>1</v>
       </c>
       <c r="M2" s="2">
-        <v>1</v>
+        <v>0.93</v>
       </c>
       <c r="N2" s="2">
-        <v>0.93</v>
+        <v>1</v>
       </c>
       <c r="O2" s="2">
         <v>1</v>
@@ -2484,10 +2486,10 @@
         <v>0</v>
       </c>
       <c r="M3" s="2">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="N3" s="2">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
       </c>
       <c r="O3" s="2">
         <v>0</v>
@@ -2685,19 +2687,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:J4">
-    <cfRule type="colorScale" priority="25">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K4">
+  <conditionalFormatting sqref="J2:J4">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -2709,7 +2699,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L4 X2:X4">
+  <conditionalFormatting sqref="K2:K4 X2:X4">
     <cfRule type="colorScale" priority="31">
       <colorScale>
         <cfvo type="min"/>
@@ -2721,7 +2711,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:N4 D2:D4 P2:P4 S2:W4">
+  <conditionalFormatting sqref="L2:M4 D2:D4 P2:P4 S2:W4">
     <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="min"/>
@@ -2817,6 +2807,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N4 H2:I4">
+    <cfRule type="colorScale" priority="34">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2837,7 +2839,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1">
         <v>1</v>
@@ -2878,7 +2880,7 @@
     </row>
     <row r="2" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
@@ -2919,7 +2921,7 @@
     </row>
     <row r="3" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B3" s="2">
         <v>1</v>
@@ -2960,7 +2962,7 @@
     </row>
     <row r="4" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" s="2">
         <v>1</v>
@@ -3001,7 +3003,7 @@
     </row>
     <row r="5" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" s="2">
         <v>1</v>
@@ -3042,7 +3044,7 @@
     </row>
     <row r="6" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B6" s="2">
         <v>1</v>
@@ -3083,7 +3085,7 @@
     </row>
     <row r="7" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
@@ -3165,7 +3167,7 @@
     </row>
     <row r="9" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B9" s="2">
         <v>1</v>
@@ -3206,19 +3208,19 @@
     </row>
     <row r="10" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="B10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" s="2">
         <v>1</v>
@@ -3233,33 +3235,33 @@
         <v>1</v>
       </c>
       <c r="J10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="B11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="2">
         <v>1</v>
@@ -3274,21 +3276,21 @@
         <v>1</v>
       </c>
       <c r="J11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="B12" s="2">
         <v>1</v>
@@ -3329,7 +3331,7 @@
     </row>
     <row r="13" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="B13" s="2">
         <v>1</v>
@@ -3370,7 +3372,7 @@
     </row>
     <row r="14" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="B14" s="2">
         <v>1</v>
@@ -3411,7 +3413,7 @@
     </row>
     <row r="15" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B15" s="2">
         <v>1</v>
@@ -3452,7 +3454,7 @@
     </row>
     <row r="16" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" s="2">
         <v>1</v>
@@ -3493,7 +3495,7 @@
     </row>
     <row r="17" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B17" s="2">
         <v>1</v>
@@ -3534,7 +3536,7 @@
     </row>
     <row r="18" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" s="2">
         <v>1</v>
@@ -3575,7 +3577,7 @@
     </row>
     <row r="19" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" s="2">
         <v>1</v>
@@ -3616,7 +3618,7 @@
     </row>
     <row r="20" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B20" s="2">
         <v>1</v>
@@ -3657,7 +3659,7 @@
     </row>
     <row r="21" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B21" s="2">
         <v>1</v>
@@ -3698,7 +3700,7 @@
     </row>
     <row r="22" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B22" s="2">
         <v>1</v>
@@ -3780,7 +3782,7 @@
     </row>
     <row r="24" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B24" s="2">
         <v>1</v>
@@ -3821,7 +3823,7 @@
     </row>
     <row r="25" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B25" s="2">
         <v>1</v>
@@ -3862,7 +3864,7 @@
     </row>
     <row r="26" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B26" s="2">
         <v>1</v>
@@ -3903,7 +3905,7 @@
     </row>
     <row r="27" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B27" s="2">
         <v>1</v>
@@ -3944,7 +3946,7 @@
     </row>
     <row r="28" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B28" s="2">
         <v>1</v>
@@ -4026,7 +4028,7 @@
     </row>
     <row r="30" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="2">
         <v>1</v>
@@ -4067,7 +4069,7 @@
     </row>
     <row r="31" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B31" s="2">
         <v>1</v>
@@ -4108,7 +4110,7 @@
     </row>
     <row r="32" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32" s="2">
         <v>1</v>
@@ -4192,18 +4194,6 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M27">
     <sortCondition ref="A2:A27"/>
   </sortState>
-  <conditionalFormatting sqref="B2:M8 B10:M27">
-    <cfRule type="colorScale" priority="32">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B9:M9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -4252,6 +4242,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B10:M27 B2:M8">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Upload boiler functions for load emulator v2
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/files/energy/input/load_emulator/input_emulator_v2/0. metadata_load_emulator_v2.xlsx
+++ b/files/energy/input/load_emulator/input_emulator_v2/0. metadata_load_emulator_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rsericerca-my.sharepoint.com/personal/rollo_rse-web_it/Documents/Desktop/CACER simulator - public repo/CACER-simulator/files/energy/input/load_emulator/input_emulator_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1049" documentId="11_F25DC773A252ABDACC1048A8291C5FB25ADE58F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA854FAF-612B-4940-B249-A39C593B9573}"/>
+  <xr:revisionPtr revIDLastSave="1054" documentId="11_F25DC773A252ABDACC1048A8291C5FB25ADE58F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEFADAC6-DA1F-4FF1-9593-0DA99C7CA460}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="708" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="708" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clusters_distribution" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Dati Istat</t>
+    Dati Istat -&gt; 20%</t>
       </text>
     </comment>
     <comment ref="E1" authorId="1" shapeId="0" xr:uid="{D4D25116-92E2-4F78-8010-BF7F1BD55086}">
@@ -692,7 +692,7 @@
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="C1" dT="2026-03-24T14:25:52.95" personId="{776CA3F5-2BE0-4A02-A953-A7EBF94F0315}" id="{18778F8A-622C-4A32-A415-510A6BEF5C4A}">
-    <text>Dati Istat</text>
+    <text>Dati Istat -&gt; 20%</text>
   </threadedComment>
   <threadedComment ref="E1" dT="2026-03-24T15:06:30.26" personId="{776CA3F5-2BE0-4A02-A953-A7EBF94F0315}" id="{D4D25116-92E2-4F78-8010-BF7F1BD55086}">
     <text>Information no available: fixed value</text>
@@ -2713,6 +2713,18 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:M4 D2:D4 P2:P4 S2:W4">
     <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N4 H2:I4">
+    <cfRule type="colorScale" priority="34">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -2807,18 +2819,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N4 H2:I4">
-    <cfRule type="colorScale" priority="34">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4196,6 +4196,18 @@
   </sortState>
   <conditionalFormatting sqref="B9:M9">
     <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10:M27 B2:M8">
+    <cfRule type="colorScale" priority="33">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4242,18 +4254,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B10:M27 B2:M8">
-    <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updating load emulator v2: blnp profiles corrected and modified boiler simulation
</commit_message>
<xml_diff>
--- a/files/energy/input/load_emulator/input_emulator_v2/0. metadata_load_emulator_v2.xlsx
+++ b/files/energy/input/load_emulator/input_emulator_v2/0. metadata_load_emulator_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rsericerca-my.sharepoint.com/personal/rollo_rse-web_it/Documents/Desktop/CACER simulator - public repo/CACER-simulator/files/energy/input/load_emulator/input_emulator_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1054" documentId="11_F25DC773A252ABDACC1048A8291C5FB25ADE58F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEFADAC6-DA1F-4FF1-9593-0DA99C7CA460}"/>
+  <xr:revisionPtr revIDLastSave="1060" documentId="11_F25DC773A252ABDACC1048A8291C5FB25ADE58F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82763478-F1B0-49E5-8ABE-DDC1AE1F3F9F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="708" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="708" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clusters_distribution" sheetId="1" r:id="rId1"/>
@@ -3135,28 +3135,28 @@
         <v>1</v>
       </c>
       <c r="D8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" s="2">
         <v>1</v>
@@ -3182,16 +3182,16 @@
         <v>1</v>
       </c>
       <c r="F9" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" s="2">
         <v>1</v>
@@ -4194,8 +4194,8 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M27">
     <sortCondition ref="A2:A27"/>
   </sortState>
-  <conditionalFormatting sqref="B9:M9">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="B9:C9">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4207,7 +4207,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:M27 B2:M8">
-    <cfRule type="colorScale" priority="33">
+    <cfRule type="colorScale" priority="38">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4219,6 +4219,42 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28:M29">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30:M31">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B32:M33">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F9:I9">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -4230,7 +4266,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B30:M31">
+  <conditionalFormatting sqref="J9:M9">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -4242,8 +4278,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B32:M33">
+  <conditionalFormatting sqref="D9:E9">
     <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:M33">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>